<commit_message>
Update app branding to Totum Talent and improve Excel report generation
- Change browser tab title from 'Lovable App' to 'Totum Talent'
- Remove favicon icon for clean branding
- Update meta tags for better SEO and social sharing
- Implement ExcelJS for Excel report generation
- Fix template loading and worksheet access
- Add ExcelJS package dependency
- Update Excel template handling for better compatibility
</commit_message>
<xml_diff>
--- a/public/templates/reporte_template.xlsx
+++ b/public/templates/reporte_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11028"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/041d57eb966b3500/Consultoría Angie-ak/Totum Talent - Procesos/Proyecto Interno - Prestaciones y Beneficios/Documentos Ejemplo/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sebastianloredo/Documents/clienthub-connect/public/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="64" documentId="8_{90A6FF4F-0B1F-4E2A-9EFB-6102E2E60465}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{87FF2A50-AF6B-4710-8E17-0DCC375DF954}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFF1CAA2-F0DD-5444-8173-AE62FFE28A11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="878" xr2:uid="{365CDAA6-48A6-4DE4-A11F-E92E427B642D}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="26140" windowHeight="14880" tabRatio="878" xr2:uid="{365CDAA6-48A6-4DE4-A11F-E92E427B642D}"/>
   </bookViews>
   <sheets>
     <sheet name="COMPETITIVIDAD" sheetId="14" r:id="rId1"/>
@@ -37,7 +37,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
@@ -47,9 +46,6 @@
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="98">
-  <si>
-    <t>ANALISIS DE COMPETITIVIDAD</t>
-  </si>
   <si>
     <t>A continuación, se muestran los resultados obtenidos del análisis de competitividad acorde a los puestos tipo seleccionados y perfiles de puesto.</t>
   </si>
@@ -603,6 +599,9 @@
   </si>
   <si>
     <t>INFORMACIÓN DEL PUESTO</t>
+  </si>
+  <si>
+    <t>ANALISIS DE COMPETITIVIDAD</t>
   </si>
 </sst>
 </file>
@@ -1107,11 +1106,20 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="24" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="18" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1125,8 +1133,8 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1134,23 +1142,14 @@
     <xf numFmtId="0" fontId="24" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="24" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="18" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="24" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1278,6 +1277,134 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="_-&quot;$&quot;* #,##0_-;\-&quot;$&quot;* #,##0_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="_-&quot;$&quot;* #,##0_-;\-&quot;$&quot;* #,##0_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="_-&quot;$&quot;* #,##0_-;\-&quot;$&quot;* #,##0_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="_-&quot;$&quot;* #,##0_-;\-&quot;$&quot;* #,##0_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color rgb="FFFFFFFF"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color theme="0"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="0"/>
+        </left>
+        <right style="thin">
+          <color theme="0"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -1556,13 +1683,6 @@
       </font>
     </dxf>
     <dxf>
-      <border>
-        <bottom style="thin">
-          <color theme="0"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <font>
         <strike val="0"/>
         <outline val="0"/>
@@ -1575,6 +1695,13 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color theme="0"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1593,134 +1720,6 @@
         <horizontal style="thin">
           <color theme="0"/>
         </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="_-&quot;$&quot;* #,##0_-;\-&quot;$&quot;* #,##0_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="_-&quot;$&quot;* #,##0_-;\-&quot;$&quot;* #,##0_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="_-&quot;$&quot;* #,##0_-;\-&quot;$&quot;* #,##0_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="_-&quot;$&quot;* #,##0_-;\-&quot;$&quot;* #,##0_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color rgb="FFFFFFFF"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="9"/>
-        <color theme="0"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF0070C0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="0"/>
-        </left>
-        <right style="thin">
-          <color theme="0"/>
-        </right>
-        <top/>
-        <bottom/>
       </border>
     </dxf>
   </dxfs>
@@ -1747,122 +1746,11 @@
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="absolute">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>229228</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>6132</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>88695</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Imagen 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C05429F9-DD81-4615-9F46-9DB3EC7FEEBB}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="419100" y="259080"/>
-          <a:ext cx="2039373" cy="378255"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="absolute">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>267277</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>59452</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>1557037</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>71947</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Imagen 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{438DEDE3-4209-414A-89A7-3C2E1EBE8089}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="267277" y="242332"/>
-          <a:ext cx="2013305" cy="378255"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <xxl21:alternateUrls>
       <xxl21:absoluteUrl r:id="rId2"/>
-      <xxl21:relativeUrl r:id="rId3"/>
     </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Hoja1"/>
@@ -1901,7 +1789,6 @@
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <xxl21:alternateUrls>
       <xxl21:absoluteUrl r:id="rId2"/>
-      <xxl21:relativeUrl r:id="rId3"/>
     </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Instrucciones"/>
@@ -1922,19 +1809,19 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{87A49776-68A0-43B5-BB1E-A16B09B37AFF}" name="Tabla14" displayName="Tabla14" ref="B22:I42" totalsRowShown="0" headerRowDxfId="26" dataDxfId="25" headerRowBorderDxfId="24">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{87A49776-68A0-43B5-BB1E-A16B09B37AFF}" name="Tabla14" displayName="Tabla14" ref="B22:I42" totalsRowShown="0" headerRowDxfId="34" dataDxfId="32" headerRowBorderDxfId="33">
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B23:I42">
     <sortCondition ref="B22:B42"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{D12708C8-0E7A-49C4-AF57-49FDA6D85361}" name="#" dataDxfId="23"/>
-    <tableColumn id="4" xr3:uid="{A802944B-3D80-4C7E-8B64-2D7E70A9C32A}" name="ÁREA " dataDxfId="22"/>
-    <tableColumn id="2" xr3:uid="{2AE08525-3ADD-48DA-8FFD-4810875A1CA6}" name="PUESTOS " dataDxfId="21"/>
-    <tableColumn id="9" xr3:uid="{3CCE85D7-562D-4311-8672-072C99DC8837}" name="25P" dataDxfId="20"/>
-    <tableColumn id="10" xr3:uid="{45C0FECB-2BC9-4DD0-86D9-5419EAE36720}" name="50P" dataDxfId="19"/>
-    <tableColumn id="11" xr3:uid="{3CC8069E-17AC-463B-A81F-4672CFF068BF}" name="PROMEDIO" dataDxfId="18"/>
-    <tableColumn id="12" xr3:uid="{870B44C8-19C3-436A-A868-6EDDEF8E9C39}" name="75P" dataDxfId="17"/>
-    <tableColumn id="14" xr3:uid="{53CDD169-AA34-4ACD-BA20-9B53A98E199E}" name="VARIANZA EN MERCADO" dataDxfId="16" dataCellStyle="Porcentaje">
+    <tableColumn id="1" xr3:uid="{D12708C8-0E7A-49C4-AF57-49FDA6D85361}" name="#" dataDxfId="31"/>
+    <tableColumn id="4" xr3:uid="{A802944B-3D80-4C7E-8B64-2D7E70A9C32A}" name="ÁREA " dataDxfId="30"/>
+    <tableColumn id="2" xr3:uid="{2AE08525-3ADD-48DA-8FFD-4810875A1CA6}" name="PUESTOS " dataDxfId="29"/>
+    <tableColumn id="9" xr3:uid="{3CCE85D7-562D-4311-8672-072C99DC8837}" name="25P" dataDxfId="28"/>
+    <tableColumn id="10" xr3:uid="{45C0FECB-2BC9-4DD0-86D9-5419EAE36720}" name="50P" dataDxfId="27"/>
+    <tableColumn id="11" xr3:uid="{3CC8069E-17AC-463B-A81F-4672CFF068BF}" name="PROMEDIO" dataDxfId="26"/>
+    <tableColumn id="12" xr3:uid="{870B44C8-19C3-436A-A868-6EDDEF8E9C39}" name="75P" dataDxfId="25"/>
+    <tableColumn id="14" xr3:uid="{53CDD169-AA34-4ACD-BA20-9B53A98E199E}" name="VARIANZA EN MERCADO" dataDxfId="24" dataCellStyle="Porcentaje">
       <calculatedColumnFormula>Tabla14[[#This Row],[75P]]/Tabla14[[#This Row],[25P]]-1</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1943,16 +1830,16 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{09AD7FCA-00AC-4C47-880F-3A02FDAAB3CF}" name="Comp_total1011" displayName="Comp_total1011" ref="B55:H75" totalsRowShown="0" headerRowDxfId="34" headerRowBorderDxfId="33">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{09AD7FCA-00AC-4C47-880F-3A02FDAAB3CF}" name="Comp_total1011" displayName="Comp_total1011" ref="B55:H75" totalsRowShown="0" headerRowDxfId="23" headerRowBorderDxfId="22">
   <autoFilter ref="B55:H75" xr:uid="{09AD7FCA-00AC-4C47-880F-3A02FDAAB3CF}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{19DB1777-6E7F-4929-BF86-5E1C4F2F25EF}" name="#" dataDxfId="32"/>
-    <tableColumn id="4" xr3:uid="{E9C0BE7E-2F54-485C-82E6-A575DBDF0F84}" name="Área" dataDxfId="31"/>
+    <tableColumn id="1" xr3:uid="{19DB1777-6E7F-4929-BF86-5E1C4F2F25EF}" name="#" dataDxfId="21"/>
+    <tableColumn id="4" xr3:uid="{E9C0BE7E-2F54-485C-82E6-A575DBDF0F84}" name="Área" dataDxfId="20"/>
     <tableColumn id="2" xr3:uid="{40274BDC-950D-41C5-A041-1065D5C1E6DB}" name="Nombre de Puestos"/>
-    <tableColumn id="17" xr3:uid="{C1116185-F8A6-45D1-BBE9-1AB23F04B9F9}" name="Costo mensual actual" dataDxfId="30" dataCellStyle="Moneda"/>
-    <tableColumn id="19" xr3:uid="{B60C2DC2-3CA8-418A-BA7E-12137AB6B470}" name="Costo mensual - 25P" dataDxfId="29" dataCellStyle="Moneda"/>
-    <tableColumn id="20" xr3:uid="{A4A49F55-8FB7-49F6-9C04-5B907119A086}" name="Costo mensual - 50P" dataDxfId="28" dataCellStyle="Moneda"/>
-    <tableColumn id="23" xr3:uid="{4C99EAE2-58F9-4B40-9052-F1B810CB8F45}" name="Costo mensual - 75P" dataDxfId="27" dataCellStyle="Moneda"/>
+    <tableColumn id="17" xr3:uid="{C1116185-F8A6-45D1-BBE9-1AB23F04B9F9}" name="Costo mensual actual" dataDxfId="19" dataCellStyle="Moneda"/>
+    <tableColumn id="19" xr3:uid="{B60C2DC2-3CA8-418A-BA7E-12137AB6B470}" name="Costo mensual - 25P" dataDxfId="18" dataCellStyle="Moneda"/>
+    <tableColumn id="20" xr3:uid="{A4A49F55-8FB7-49F6-9C04-5B907119A086}" name="Costo mensual - 50P" dataDxfId="17" dataCellStyle="Moneda"/>
+    <tableColumn id="23" xr3:uid="{4C99EAE2-58F9-4B40-9052-F1B810CB8F45}" name="Costo mensual - 75P" dataDxfId="16" dataCellStyle="Moneda"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2300,154 +2187,155 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4852433D-E10A-4FCD-89E4-FBEB63F93038}">
   <dimension ref="A1:U66"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="0" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="0" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="2.88671875" customWidth="1"/>
-    <col min="2" max="2" width="4.5546875" customWidth="1"/>
+    <col min="1" max="1" width="2.83203125" customWidth="1"/>
+    <col min="2" max="2" width="4.5" customWidth="1"/>
     <col min="3" max="3" width="28.33203125" customWidth="1"/>
-    <col min="4" max="4" width="32.5546875" customWidth="1"/>
-    <col min="5" max="9" width="15.21875" customWidth="1"/>
-    <col min="10" max="11" width="11.88671875" customWidth="1"/>
-    <col min="12" max="12" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="32.5" customWidth="1"/>
+    <col min="5" max="9" width="15.1640625" customWidth="1"/>
+    <col min="10" max="11" width="11.83203125" customWidth="1"/>
+    <col min="12" max="12" width="12.5" bestFit="1" customWidth="1"/>
     <col min="13" max="14" width="4.6640625" customWidth="1"/>
-    <col min="15" max="15" width="4.6640625" hidden="1"/>
-    <col min="22" max="16384" width="11.5546875" hidden="1"/>
+    <col min="15" max="15" width="4.6640625" hidden="1" customWidth="1"/>
+    <col min="16" max="21" width="0" hidden="1" customWidth="1"/>
+    <col min="22" max="16384" width="11.5" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:11" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:11" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="2:11" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="4" spans="2:11" ht="47.4" x14ac:dyDescent="0.9">
-      <c r="B4" s="54" t="s">
+    <row r="1" spans="2:11" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="2:11" x14ac:dyDescent="0.2"/>
+    <row r="3" spans="2:11" x14ac:dyDescent="0.2"/>
+    <row r="4" spans="2:11" ht="47" x14ac:dyDescent="0.55000000000000004">
+      <c r="B4" s="53" t="s">
+        <v>97</v>
+      </c>
+      <c r="C4" s="53"/>
+      <c r="D4" s="53"/>
+      <c r="E4" s="53"/>
+      <c r="F4" s="53"/>
+      <c r="G4" s="53"/>
+      <c r="H4" s="53"/>
+      <c r="I4" s="53"/>
+      <c r="J4" s="53"/>
+      <c r="K4" s="53"/>
+    </row>
+    <row r="5" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B5" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="54"/>
-      <c r="D4" s="54"/>
-      <c r="E4" s="54"/>
-      <c r="F4" s="54"/>
-      <c r="G4" s="54"/>
-      <c r="H4" s="54"/>
-      <c r="I4" s="54"/>
-      <c r="J4" s="54"/>
-      <c r="K4" s="54"/>
-    </row>
-    <row r="5" spans="2:11" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="B5" s="7" t="s">
+    </row>
+    <row r="6" spans="2:11" x14ac:dyDescent="0.2"/>
+    <row r="7" spans="2:11" ht="23" x14ac:dyDescent="0.25">
+      <c r="B7" s="4" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="2:11" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="7" spans="2:11" ht="27.6" x14ac:dyDescent="0.65">
-      <c r="B7" s="4" t="s">
+    <row r="8" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B8" s="5" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="2:11" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="B8" s="5" t="s">
+    <row r="9" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B9" s="6" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="2:11" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="B9" s="6" t="s">
+    <row r="10" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B10" s="6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="2:11" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="B10" s="6" t="s">
+    <row r="11" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B11" s="6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="2:11" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="B11" s="6" t="s">
+    <row r="12" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B12" s="6" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="2:11" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="B12" s="6" t="s">
+    <row r="13" spans="2:11" x14ac:dyDescent="0.2"/>
+    <row r="14" spans="2:11" s="28" customFormat="1" ht="23" x14ac:dyDescent="0.25">
+      <c r="B14" s="29" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="2:11" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="14" spans="2:11" s="28" customFormat="1" ht="27.6" x14ac:dyDescent="0.65">
-      <c r="B14" s="29" t="s">
+    <row r="15" spans="2:11" x14ac:dyDescent="0.2"/>
+    <row r="16" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B16" s="30" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="15" spans="2:11" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="16" spans="2:11" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="B16" s="30" t="s">
-        <v>9</v>
-      </c>
       <c r="C16" s="7"/>
     </row>
-    <row r="17" spans="2:9" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="17" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B17" s="8"/>
       <c r="C17" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="18" spans="2:9" ht="16.8" x14ac:dyDescent="0.4">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="18" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B18" s="9"/>
       <c r="C18" s="1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="19" spans="2:9" ht="16.8" x14ac:dyDescent="0.4">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B19" s="10"/>
       <c r="C19" s="1" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="20" spans="2:9" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="21" spans="2:9" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="67" t="s">
-        <v>97</v>
-      </c>
-      <c r="C21" s="67"/>
-      <c r="D21" s="67"/>
-      <c r="E21" s="67" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="20" spans="2:9" x14ac:dyDescent="0.2"/>
+    <row r="21" spans="2:9" ht="30.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B21" s="54" t="s">
+        <v>96</v>
+      </c>
+      <c r="C21" s="54"/>
+      <c r="D21" s="54"/>
+      <c r="E21" s="54" t="s">
+        <v>9</v>
+      </c>
+      <c r="F21" s="54"/>
+      <c r="G21" s="54"/>
+      <c r="H21" s="54"/>
+      <c r="I21" s="54"/>
+    </row>
+    <row r="22" spans="2:9" ht="30" x14ac:dyDescent="0.2">
+      <c r="B22" s="38" t="s">
         <v>10</v>
       </c>
-      <c r="F21" s="67"/>
-      <c r="G21" s="67"/>
-      <c r="H21" s="67"/>
-      <c r="I21" s="67"/>
-    </row>
-    <row r="22" spans="2:9" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="B22" s="38" t="s">
+      <c r="C22" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="C22" s="38" t="s">
+      <c r="D22" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="D22" s="38" t="s">
+      <c r="E22" s="43" t="s">
         <v>13</v>
       </c>
-      <c r="E22" s="43" t="s">
+      <c r="F22" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="F22" s="44" t="s">
+      <c r="G22" s="44" t="s">
         <v>15</v>
       </c>
-      <c r="G22" s="44" t="s">
+      <c r="H22" s="44" t="s">
         <v>16</v>
       </c>
-      <c r="H22" s="44" t="s">
+      <c r="I22" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="I22" s="39" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="23" spans="2:9" ht="14.4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="23" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B23" s="40">
         <v>1</v>
       </c>
       <c r="C23" s="41" t="s">
+        <v>18</v>
+      </c>
+      <c r="D23" s="41" t="s">
         <v>19</v>
-      </c>
-      <c r="D23" s="41" t="s">
-        <v>20</v>
       </c>
       <c r="E23" s="45">
         <v>135837</v>
@@ -2466,15 +2354,15 @@
         <v>0.50617283950617287</v>
       </c>
     </row>
-    <row r="24" spans="2:9" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B24" s="40">
         <v>2</v>
       </c>
       <c r="C24" s="41" t="s">
+        <v>20</v>
+      </c>
+      <c r="D24" s="40" t="s">
         <v>21</v>
-      </c>
-      <c r="D24" s="40" t="s">
-        <v>22</v>
       </c>
       <c r="E24" s="45">
         <v>128160</v>
@@ -2493,15 +2381,15 @@
         <v>0.348314606741573</v>
       </c>
     </row>
-    <row r="25" spans="2:9" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B25" s="40">
         <v>3</v>
       </c>
       <c r="C25" s="41" t="s">
+        <v>22</v>
+      </c>
+      <c r="D25" s="40" t="s">
         <v>23</v>
-      </c>
-      <c r="D25" s="40" t="s">
-        <v>24</v>
       </c>
       <c r="E25" s="45">
         <v>87516</v>
@@ -2520,15 +2408,15 @@
         <v>0.40909090909090917</v>
       </c>
     </row>
-    <row r="26" spans="2:9" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B26" s="40">
         <v>4</v>
       </c>
       <c r="C26" s="41" t="s">
+        <v>24</v>
+      </c>
+      <c r="D26" s="40" t="s">
         <v>25</v>
-      </c>
-      <c r="D26" s="40" t="s">
-        <v>26</v>
       </c>
       <c r="E26" s="45">
         <v>76950</v>
@@ -2547,15 +2435,15 @@
         <v>0.58024691358024683</v>
       </c>
     </row>
-    <row r="27" spans="2:9" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B27" s="40">
         <v>5</v>
       </c>
       <c r="C27" s="41" t="s">
+        <v>26</v>
+      </c>
+      <c r="D27" s="40" t="s">
         <v>27</v>
-      </c>
-      <c r="D27" s="40" t="s">
-        <v>28</v>
       </c>
       <c r="E27" s="45">
         <v>89880</v>
@@ -2574,15 +2462,15 @@
         <v>0.52380952380952372</v>
       </c>
     </row>
-    <row r="28" spans="2:9" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B28" s="40">
         <v>6</v>
       </c>
       <c r="C28" s="40" t="s">
+        <v>28</v>
+      </c>
+      <c r="D28" s="40" t="s">
         <v>29</v>
-      </c>
-      <c r="D28" s="40" t="s">
-        <v>30</v>
       </c>
       <c r="E28" s="45">
         <v>38304.5</v>
@@ -2601,15 +2489,15 @@
         <v>0.44578313253012047</v>
       </c>
     </row>
-    <row r="29" spans="2:9" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B29" s="40">
         <v>7</v>
       </c>
       <c r="C29" s="40" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D29" s="41" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E29" s="45">
         <v>30651.600000000002</v>
@@ -2628,15 +2516,15 @@
         <v>0.37078651685393238</v>
       </c>
     </row>
-    <row r="30" spans="2:9" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B30" s="40">
         <v>8</v>
       </c>
       <c r="C30" s="40" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D30" s="40" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E30" s="45">
         <v>47749.5</v>
@@ -2655,15 +2543,15 @@
         <v>0.53086419753086411</v>
       </c>
     </row>
-    <row r="31" spans="2:9" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B31" s="40">
         <v>9</v>
       </c>
       <c r="C31" s="40" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D31" s="40" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E31" s="45">
         <v>39060</v>
@@ -2682,15 +2570,15 @@
         <v>0.48809523809523814</v>
       </c>
     </row>
-    <row r="32" spans="2:9" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B32" s="40">
         <v>10</v>
       </c>
       <c r="C32" s="40" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D32" s="40" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E32" s="45">
         <v>19008</v>
@@ -2709,15 +2597,15 @@
         <v>0.625</v>
       </c>
     </row>
-    <row r="33" spans="2:9" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B33" s="40">
         <v>11</v>
       </c>
       <c r="C33" s="40" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D33" s="40" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E33" s="45">
         <v>14968.8</v>
@@ -2736,15 +2624,15 @@
         <v>0.48809523809523814</v>
       </c>
     </row>
-    <row r="34" spans="2:9" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B34" s="40">
         <v>12</v>
       </c>
       <c r="C34" s="40" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D34" s="40" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E34" s="45">
         <v>19575</v>
@@ -2763,15 +2651,15 @@
         <v>0.4137931034482758</v>
       </c>
     </row>
-    <row r="35" spans="2:9" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B35" s="40">
         <v>13</v>
       </c>
       <c r="C35" s="40" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D35" s="40" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E35" s="45">
         <v>24731.199999999997</v>
@@ -2790,15 +2678,15 @@
         <v>0.48780487804878048</v>
       </c>
     </row>
-    <row r="36" spans="2:9" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B36" s="40">
         <v>14</v>
       </c>
       <c r="C36" s="40" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D36" s="40" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E36" s="45">
         <v>8017.7999999999993</v>
@@ -2817,15 +2705,15 @@
         <v>0.55421686746987953</v>
       </c>
     </row>
-    <row r="37" spans="2:9" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B37" s="40">
         <v>15</v>
       </c>
       <c r="C37" s="40" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D37" s="40" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E37" s="45">
         <v>10137.6</v>
@@ -2844,15 +2732,15 @@
         <v>0.38636363636363624</v>
       </c>
     </row>
-    <row r="38" spans="2:9" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B38" s="40">
         <v>16</v>
       </c>
       <c r="C38" s="40" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D38" s="40" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E38" s="45">
         <v>23800.000000000004</v>
@@ -2871,15 +2759,15 @@
         <v>0.49411764705882355</v>
       </c>
     </row>
-    <row r="39" spans="2:9" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B39" s="40">
         <v>17</v>
       </c>
       <c r="C39" s="40" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D39" s="40" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E39" s="45">
         <v>19197</v>
@@ -2898,15 +2786,15 @@
         <v>0.5185185185185186</v>
       </c>
     </row>
-    <row r="40" spans="2:9" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B40" s="40">
         <v>18</v>
       </c>
       <c r="C40" s="40" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D40" s="40" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E40" s="45">
         <v>34800</v>
@@ -2925,15 +2813,15 @@
         <v>0.43678160919540221</v>
       </c>
     </row>
-    <row r="41" spans="2:9" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B41" s="40">
         <v>19</v>
       </c>
       <c r="C41" s="40" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D41" s="40" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E41" s="45">
         <v>32894.400000000001</v>
@@ -2952,15 +2840,15 @@
         <v>0.46590909090909105</v>
       </c>
     </row>
-    <row r="42" spans="2:9" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B42" s="40">
         <v>20</v>
       </c>
       <c r="C42" s="40" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D42" s="40" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E42" s="45">
         <v>15470</v>
@@ -2979,30 +2867,30 @@
         <v>0.51764705882352935</v>
       </c>
     </row>
-    <row r="43" spans="2:9" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="44" spans="2:9" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="45" spans="2:9" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="46" spans="2:9" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="47" spans="2:9" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="48" spans="2:9" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="49" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="50" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="51" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="52" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="53" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="54" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="55" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="56" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="57" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="58" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="59" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="60" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="61" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="62" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="63" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="64" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="65" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="66" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="43" spans="2:9" x14ac:dyDescent="0.2"/>
+    <row r="44" spans="2:9" x14ac:dyDescent="0.2"/>
+    <row r="45" spans="2:9" x14ac:dyDescent="0.2"/>
+    <row r="46" spans="2:9" x14ac:dyDescent="0.2"/>
+    <row r="47" spans="2:9" x14ac:dyDescent="0.2"/>
+    <row r="48" spans="2:9" x14ac:dyDescent="0.2"/>
+    <row r="49" x14ac:dyDescent="0.2"/>
+    <row r="50" x14ac:dyDescent="0.2"/>
+    <row r="51" x14ac:dyDescent="0.2"/>
+    <row r="52" x14ac:dyDescent="0.2"/>
+    <row r="53" x14ac:dyDescent="0.2"/>
+    <row r="54" x14ac:dyDescent="0.2"/>
+    <row r="55" x14ac:dyDescent="0.2"/>
+    <row r="56" x14ac:dyDescent="0.2"/>
+    <row r="57" x14ac:dyDescent="0.2"/>
+    <row r="58" x14ac:dyDescent="0.2"/>
+    <row r="59" x14ac:dyDescent="0.2"/>
+    <row r="60" x14ac:dyDescent="0.2"/>
+    <row r="61" x14ac:dyDescent="0.2"/>
+    <row r="62" x14ac:dyDescent="0.2"/>
+    <row r="63" x14ac:dyDescent="0.2"/>
+    <row r="64" x14ac:dyDescent="0.2"/>
+    <row r="65" x14ac:dyDescent="0.2"/>
+    <row r="66" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="B4:K4"/>
@@ -3011,9 +2899,8 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
-  <drawing r:id="rId2"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
@@ -3021,215 +2908,215 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CBD840F8-6B73-4F62-9C0E-29FB77B2FE9B}">
   <dimension ref="B1:AT175"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="5.109375" customWidth="1"/>
-    <col min="2" max="2" width="5.44140625" customWidth="1"/>
+    <col min="1" max="1" width="5.1640625" customWidth="1"/>
+    <col min="2" max="2" width="5.5" customWidth="1"/>
     <col min="3" max="3" width="23.33203125" customWidth="1"/>
-    <col min="4" max="4" width="30.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="30.83203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="13" width="17.109375" customWidth="1"/>
+    <col min="6" max="13" width="17.1640625" customWidth="1"/>
     <col min="14" max="14" width="14" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="12" customWidth="1"/>
     <col min="16" max="16" width="14.33203125" customWidth="1"/>
     <col min="17" max="29" width="14" customWidth="1"/>
-    <col min="30" max="30" width="11.5546875" customWidth="1"/>
-    <col min="31" max="31" width="12.44140625" customWidth="1"/>
+    <col min="30" max="30" width="11.5" customWidth="1"/>
+    <col min="31" max="31" width="12.5" customWidth="1"/>
     <col min="32" max="32" width="14" customWidth="1"/>
-    <col min="33" max="36" width="9.109375" customWidth="1"/>
+    <col min="33" max="36" width="9.1640625" customWidth="1"/>
     <col min="37" max="37" width="13.33203125" customWidth="1"/>
     <col min="38" max="38" width="12.33203125" customWidth="1"/>
     <col min="39" max="40" width="14.33203125" customWidth="1"/>
     <col min="41" max="43" width="14.6640625" customWidth="1"/>
-    <col min="44" max="45" width="15.109375" customWidth="1"/>
+    <col min="44" max="45" width="15.1640625" customWidth="1"/>
     <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="20.109375" customWidth="1"/>
-    <col min="48" max="50" width="11.5546875" customWidth="1"/>
+    <col min="47" max="47" width="20.1640625" customWidth="1"/>
+    <col min="48" max="50" width="11.5" customWidth="1"/>
     <col min="51" max="51" width="13" customWidth="1"/>
-    <col min="52" max="52" width="20.109375" customWidth="1"/>
-    <col min="53" max="55" width="11.5546875" customWidth="1"/>
-    <col min="56" max="56" width="16.109375" customWidth="1"/>
-    <col min="57" max="57" width="20.109375" customWidth="1"/>
-    <col min="58" max="58" width="9.109375" customWidth="1"/>
+    <col min="52" max="52" width="20.1640625" customWidth="1"/>
+    <col min="53" max="55" width="11.5" customWidth="1"/>
+    <col min="56" max="56" width="16.1640625" customWidth="1"/>
+    <col min="57" max="57" width="20.1640625" customWidth="1"/>
+    <col min="58" max="58" width="9.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:46" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:46" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="2:46" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="4" spans="2:46" ht="47.4" x14ac:dyDescent="0.9">
-      <c r="B4" s="54" t="s">
-        <v>45</v>
-      </c>
-      <c r="C4" s="54"/>
-      <c r="D4" s="54"/>
-      <c r="E4" s="54"/>
-      <c r="F4" s="54"/>
-      <c r="G4" s="54"/>
-      <c r="H4" s="54"/>
-      <c r="I4" s="54"/>
-      <c r="J4" s="54"/>
-      <c r="K4" s="54"/>
-      <c r="L4" s="54"/>
-      <c r="M4" s="54"/>
-      <c r="N4" s="54"/>
-      <c r="O4" s="54"/>
-      <c r="P4" s="54"/>
-      <c r="Q4" s="54"/>
-      <c r="R4" s="54"/>
-      <c r="S4" s="54"/>
-      <c r="T4" s="54"/>
-      <c r="U4" s="54"/>
-      <c r="V4" s="54"/>
-      <c r="W4" s="54"/>
-      <c r="X4" s="54"/>
-      <c r="Y4" s="54"/>
-      <c r="Z4" s="54"/>
-      <c r="AA4" s="54"/>
-      <c r="AB4" s="54"/>
-      <c r="AC4" s="54"/>
-      <c r="AD4" s="54"/>
-      <c r="AE4" s="54"/>
-      <c r="AF4" s="54"/>
-      <c r="AG4" s="54"/>
-      <c r="AH4" s="54"/>
-      <c r="AI4" s="54"/>
-      <c r="AJ4" s="54"/>
-      <c r="AK4" s="54"/>
-      <c r="AL4" s="54"/>
-      <c r="AM4" s="54"/>
-      <c r="AN4" s="54"/>
-      <c r="AO4" s="54"/>
+    <row r="1" spans="2:46" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="2:46" x14ac:dyDescent="0.2"/>
+    <row r="3" spans="2:46" x14ac:dyDescent="0.2"/>
+    <row r="4" spans="2:46" ht="47" x14ac:dyDescent="0.55000000000000004">
+      <c r="B4" s="53" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" s="53"/>
+      <c r="D4" s="53"/>
+      <c r="E4" s="53"/>
+      <c r="F4" s="53"/>
+      <c r="G4" s="53"/>
+      <c r="H4" s="53"/>
+      <c r="I4" s="53"/>
+      <c r="J4" s="53"/>
+      <c r="K4" s="53"/>
+      <c r="L4" s="53"/>
+      <c r="M4" s="53"/>
+      <c r="N4" s="53"/>
+      <c r="O4" s="53"/>
+      <c r="P4" s="53"/>
+      <c r="Q4" s="53"/>
+      <c r="R4" s="53"/>
+      <c r="S4" s="53"/>
+      <c r="T4" s="53"/>
+      <c r="U4" s="53"/>
+      <c r="V4" s="53"/>
+      <c r="W4" s="53"/>
+      <c r="X4" s="53"/>
+      <c r="Y4" s="53"/>
+      <c r="Z4" s="53"/>
+      <c r="AA4" s="53"/>
+      <c r="AB4" s="53"/>
+      <c r="AC4" s="53"/>
+      <c r="AD4" s="53"/>
+      <c r="AE4" s="53"/>
+      <c r="AF4" s="53"/>
+      <c r="AG4" s="53"/>
+      <c r="AH4" s="53"/>
+      <c r="AI4" s="53"/>
+      <c r="AJ4" s="53"/>
+      <c r="AK4" s="53"/>
+      <c r="AL4" s="53"/>
+      <c r="AM4" s="53"/>
+      <c r="AN4" s="53"/>
+      <c r="AO4" s="53"/>
       <c r="AP4" s="34"/>
       <c r="AQ4" s="34"/>
       <c r="AR4" s="34"/>
       <c r="AS4" s="34"/>
       <c r="AT4" s="34"/>
     </row>
-    <row r="5" spans="2:46" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:46" x14ac:dyDescent="0.2">
       <c r="B5" s="18" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="2:46" x14ac:dyDescent="0.2">
+      <c r="B6" s="18"/>
+    </row>
+    <row r="7" spans="2:46" ht="19" x14ac:dyDescent="0.25">
+      <c r="B7" s="19" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="2:46" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B6" s="18"/>
-    </row>
-    <row r="7" spans="2:46" ht="18" x14ac:dyDescent="0.35">
-      <c r="B7" s="19" t="s">
-        <v>2</v>
-      </c>
       <c r="C7" s="19"/>
     </row>
-    <row r="8" spans="2:46" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:46" x14ac:dyDescent="0.2">
       <c r="B8" s="26" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8" s="20"/>
+    </row>
+    <row r="9" spans="2:46" x14ac:dyDescent="0.2">
+      <c r="B9" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="C8" s="20"/>
-    </row>
-    <row r="9" spans="2:46" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B9" s="26" t="s">
+      <c r="C9" s="20"/>
+    </row>
+    <row r="10" spans="2:46" x14ac:dyDescent="0.2">
+      <c r="B10" s="26" t="s">
         <v>47</v>
       </c>
-      <c r="C9" s="20"/>
-    </row>
-    <row r="10" spans="2:46" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B10" s="26" t="s">
+      <c r="C10" s="20"/>
+    </row>
+    <row r="11" spans="2:46" x14ac:dyDescent="0.2">
+      <c r="B11" s="26" t="s">
         <v>48</v>
       </c>
-      <c r="C10" s="20"/>
-    </row>
-    <row r="11" spans="2:46" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B11" s="26" t="s">
+      <c r="C11" s="20"/>
+    </row>
+    <row r="12" spans="2:46" x14ac:dyDescent="0.2">
+      <c r="B12" s="27" t="s">
         <v>49</v>
       </c>
-      <c r="C11" s="20"/>
-    </row>
-    <row r="12" spans="2:46" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B12" s="27" t="s">
-        <v>50</v>
-      </c>
       <c r="C12" s="21"/>
     </row>
-    <row r="13" spans="2:46" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:46" x14ac:dyDescent="0.2">
       <c r="B13" s="22"/>
       <c r="C13" s="22"/>
     </row>
-    <row r="14" spans="2:46" ht="18" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:46" ht="19" x14ac:dyDescent="0.25">
       <c r="B14" s="19" t="s">
+        <v>50</v>
+      </c>
+      <c r="C14" s="19"/>
+    </row>
+    <row r="15" spans="2:46" x14ac:dyDescent="0.2">
+      <c r="B15" s="58" t="s">
         <v>51</v>
       </c>
-      <c r="C14" s="19"/>
-    </row>
-    <row r="15" spans="2:46" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B15" s="55" t="s">
+      <c r="C15" s="58"/>
+      <c r="D15" s="58"/>
+      <c r="E15" s="58"/>
+      <c r="F15" s="58"/>
+      <c r="G15" s="58"/>
+    </row>
+    <row r="16" spans="2:46" x14ac:dyDescent="0.2">
+      <c r="B16" s="58"/>
+      <c r="C16" s="58"/>
+      <c r="D16" s="58"/>
+      <c r="E16" s="58"/>
+      <c r="F16" s="58"/>
+      <c r="G16" s="58"/>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B17" s="58"/>
+      <c r="C17" s="58"/>
+      <c r="D17" s="58"/>
+      <c r="E17" s="58"/>
+      <c r="F17" s="58"/>
+      <c r="G17" s="58"/>
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B18" s="58"/>
+      <c r="C18" s="58"/>
+      <c r="D18" s="58"/>
+      <c r="E18" s="58"/>
+      <c r="F18" s="58"/>
+      <c r="G18" s="58"/>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B19" s="58"/>
+      <c r="C19" s="58"/>
+      <c r="D19" s="58"/>
+      <c r="E19" s="58"/>
+      <c r="F19" s="58"/>
+      <c r="G19" s="58"/>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B20" s="59" t="s">
         <v>52</v>
       </c>
-      <c r="C15" s="55"/>
-      <c r="D15" s="55"/>
-      <c r="E15" s="55"/>
-      <c r="F15" s="55"/>
-      <c r="G15" s="55"/>
-    </row>
-    <row r="16" spans="2:46" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B16" s="55"/>
-      <c r="C16" s="55"/>
-      <c r="D16" s="55"/>
-      <c r="E16" s="55"/>
-      <c r="F16" s="55"/>
-      <c r="G16" s="55"/>
-    </row>
-    <row r="17" spans="2:7" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B17" s="55"/>
-      <c r="C17" s="55"/>
-      <c r="D17" s="55"/>
-      <c r="E17" s="55"/>
-      <c r="F17" s="55"/>
-      <c r="G17" s="55"/>
-    </row>
-    <row r="18" spans="2:7" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B18" s="55"/>
-      <c r="C18" s="55"/>
-      <c r="D18" s="55"/>
-      <c r="E18" s="55"/>
-      <c r="F18" s="55"/>
-      <c r="G18" s="55"/>
-    </row>
-    <row r="19" spans="2:7" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B19" s="55"/>
-      <c r="C19" s="55"/>
-      <c r="D19" s="55"/>
-      <c r="E19" s="55"/>
-      <c r="F19" s="55"/>
-      <c r="G19" s="55"/>
-    </row>
-    <row r="20" spans="2:7" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B20" s="56" t="s">
+      <c r="C20" s="59"/>
+      <c r="D20" s="59"/>
+      <c r="E20" s="59"/>
+      <c r="F20" s="59"/>
+      <c r="G20" s="59"/>
+    </row>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B21" s="59"/>
+      <c r="C21" s="59"/>
+      <c r="D21" s="59"/>
+      <c r="E21" s="59"/>
+      <c r="F21" s="59"/>
+      <c r="G21" s="59"/>
+    </row>
+    <row r="22" spans="2:7" x14ac:dyDescent="0.2"/>
+    <row r="23" spans="2:7" x14ac:dyDescent="0.2"/>
+    <row r="24" spans="2:7" ht="19" x14ac:dyDescent="0.25">
+      <c r="B24" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="C20" s="56"/>
-      <c r="D20" s="56"/>
-      <c r="E20" s="56"/>
-      <c r="F20" s="56"/>
-      <c r="G20" s="56"/>
-    </row>
-    <row r="21" spans="2:7" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B21" s="56"/>
-      <c r="C21" s="56"/>
-      <c r="D21" s="56"/>
-      <c r="E21" s="56"/>
-      <c r="F21" s="56"/>
-      <c r="G21" s="56"/>
-    </row>
-    <row r="22" spans="2:7" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="23" spans="2:7" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="24" spans="2:7" ht="18" x14ac:dyDescent="0.35">
-      <c r="B24" s="19" t="s">
+      <c r="C24" s="19"/>
+    </row>
+    <row r="25" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B25" s="23" t="s">
         <v>54</v>
-      </c>
-      <c r="C24" s="19"/>
-    </row>
-    <row r="25" spans="2:7" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B25" s="23" t="s">
-        <v>55</v>
       </c>
       <c r="C25" s="24"/>
       <c r="D25" s="24"/>
@@ -3237,207 +3124,207 @@
       <c r="F25" s="24"/>
       <c r="G25" s="24"/>
     </row>
-    <row r="26" spans="2:7" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B26" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="27" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B27" s="60" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="27" spans="2:7" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B27" s="57" t="s">
-        <v>57</v>
-      </c>
-      <c r="C27" s="57"/>
-      <c r="D27" s="57"/>
-      <c r="E27" s="57"/>
-      <c r="F27" s="57"/>
-      <c r="G27" s="57"/>
-    </row>
-    <row r="28" spans="2:7" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B28" s="57"/>
-      <c r="C28" s="57"/>
-      <c r="D28" s="57"/>
-      <c r="E28" s="57"/>
-      <c r="F28" s="57"/>
-      <c r="G28" s="57"/>
-    </row>
-    <row r="29" spans="2:7" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C27" s="60"/>
+      <c r="D27" s="60"/>
+      <c r="E27" s="60"/>
+      <c r="F27" s="60"/>
+      <c r="G27" s="60"/>
+    </row>
+    <row r="28" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B28" s="60"/>
+      <c r="C28" s="60"/>
+      <c r="D28" s="60"/>
+      <c r="E28" s="60"/>
+      <c r="F28" s="60"/>
+      <c r="G28" s="60"/>
+    </row>
+    <row r="29" spans="2:7" x14ac:dyDescent="0.2">
       <c r="C29" s="11"/>
       <c r="D29" s="11"/>
       <c r="E29" s="11"/>
       <c r="F29" s="11"/>
       <c r="G29" s="11"/>
     </row>
-    <row r="30" spans="2:7" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B30" s="58" t="s">
+    <row r="30" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B30" s="61" t="s">
+        <v>57</v>
+      </c>
+      <c r="C30" s="61"/>
+      <c r="D30" s="61"/>
+      <c r="E30" s="61"/>
+      <c r="F30" s="61"/>
+      <c r="G30" s="61"/>
+    </row>
+    <row r="31" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B31" s="61"/>
+      <c r="C31" s="61"/>
+      <c r="D31" s="61"/>
+      <c r="E31" s="61"/>
+      <c r="F31" s="61"/>
+      <c r="G31" s="61"/>
+    </row>
+    <row r="32" spans="2:7" x14ac:dyDescent="0.2"/>
+    <row r="33" spans="2:32" x14ac:dyDescent="0.2">
+      <c r="B33" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="C30" s="58"/>
-      <c r="D30" s="58"/>
-      <c r="E30" s="58"/>
-      <c r="F30" s="58"/>
-      <c r="G30" s="58"/>
-    </row>
-    <row r="31" spans="2:7" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B31" s="58"/>
-      <c r="C31" s="58"/>
-      <c r="D31" s="58"/>
-      <c r="E31" s="58"/>
-      <c r="F31" s="58"/>
-      <c r="G31" s="58"/>
-    </row>
-    <row r="32" spans="2:7" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="33" spans="2:32" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B33" s="12" t="s">
+      <c r="C33" s="13"/>
+    </row>
+    <row r="34" spans="2:32" x14ac:dyDescent="0.2">
+      <c r="B34" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="C33" s="13"/>
-    </row>
-    <row r="34" spans="2:32" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B34" s="14" t="s">
+      <c r="C34" s="14"/>
+    </row>
+    <row r="35" spans="2:32" x14ac:dyDescent="0.2"/>
+    <row r="36" spans="2:32" x14ac:dyDescent="0.2">
+      <c r="B36" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="C34" s="14"/>
-    </row>
-    <row r="35" spans="2:32" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="36" spans="2:32" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B36" s="12" t="s">
+      <c r="C36" s="13"/>
+    </row>
+    <row r="37" spans="2:32" x14ac:dyDescent="0.2">
+      <c r="B37" s="55" t="s">
         <v>61</v>
       </c>
-      <c r="C36" s="13"/>
-    </row>
-    <row r="37" spans="2:32" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B37" s="59" t="s">
+      <c r="C37" s="55"/>
+      <c r="D37" s="55"/>
+      <c r="E37" s="55"/>
+      <c r="F37" s="55"/>
+      <c r="G37" s="55"/>
+    </row>
+    <row r="38" spans="2:32" x14ac:dyDescent="0.2"/>
+    <row r="39" spans="2:32" x14ac:dyDescent="0.2">
+      <c r="B39" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="C37" s="59"/>
-      <c r="D37" s="59"/>
-      <c r="E37" s="59"/>
-      <c r="F37" s="59"/>
-      <c r="G37" s="59"/>
-    </row>
-    <row r="38" spans="2:32" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="39" spans="2:32" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B39" s="12" t="s">
+      <c r="C39" s="13"/>
+    </row>
+    <row r="40" spans="2:32" x14ac:dyDescent="0.2">
+      <c r="B40" s="55" t="s">
         <v>63</v>
       </c>
-      <c r="C39" s="13"/>
-    </row>
-    <row r="40" spans="2:32" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B40" s="59" t="s">
-        <v>64</v>
-      </c>
-      <c r="C40" s="59"/>
-      <c r="D40" s="59"/>
-      <c r="E40" s="59"/>
-      <c r="F40" s="59"/>
-      <c r="G40" s="59"/>
-    </row>
-    <row r="41" spans="2:32" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B41" s="59"/>
-      <c r="C41" s="59"/>
-      <c r="D41" s="59"/>
-      <c r="E41" s="59"/>
-      <c r="F41" s="59"/>
-      <c r="G41" s="59"/>
-    </row>
-    <row r="42" spans="2:32" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="43" spans="2:32" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C40" s="55"/>
+      <c r="D40" s="55"/>
+      <c r="E40" s="55"/>
+      <c r="F40" s="55"/>
+      <c r="G40" s="55"/>
+    </row>
+    <row r="41" spans="2:32" x14ac:dyDescent="0.2">
+      <c r="B41" s="55"/>
+      <c r="C41" s="55"/>
+      <c r="D41" s="55"/>
+      <c r="E41" s="55"/>
+      <c r="F41" s="55"/>
+      <c r="G41" s="55"/>
+    </row>
+    <row r="42" spans="2:32" x14ac:dyDescent="0.2"/>
+    <row r="43" spans="2:32" x14ac:dyDescent="0.2">
       <c r="AE43" s="35"/>
       <c r="AF43" s="35"/>
     </row>
-    <row r="44" spans="2:32" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:32" x14ac:dyDescent="0.2">
       <c r="AE44" s="35"/>
       <c r="AF44" s="35"/>
     </row>
-    <row r="45" spans="2:32" s="28" customFormat="1" ht="27.6" x14ac:dyDescent="0.65">
+    <row r="45" spans="2:32" s="28" customFormat="1" ht="23" x14ac:dyDescent="0.25">
       <c r="B45" s="29" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="46" spans="2:32" ht="14.4" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="46" spans="2:32" x14ac:dyDescent="0.2">
       <c r="AE46" s="35"/>
       <c r="AF46" s="35"/>
     </row>
-    <row r="47" spans="2:32" ht="23.4" x14ac:dyDescent="0.45">
+    <row r="47" spans="2:32" ht="24" x14ac:dyDescent="0.3">
       <c r="B47" s="25" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AE47" s="35"/>
       <c r="AF47" s="35"/>
     </row>
-    <row r="49" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B49" s="52" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C49" s="1"/>
       <c r="D49" s="37"/>
     </row>
-    <row r="50" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B50" s="46"/>
-      <c r="C50" s="65" t="s">
+      <c r="C50" s="56" t="s">
+        <v>93</v>
+      </c>
+      <c r="D50" s="57"/>
+    </row>
+    <row r="51" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B51" s="15"/>
+      <c r="C51" s="56" t="s">
         <v>94</v>
       </c>
-      <c r="D50" s="66"/>
-    </row>
-    <row r="51" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B51" s="15"/>
-      <c r="C51" s="65" t="s">
+      <c r="D51" s="57"/>
+    </row>
+    <row r="52" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B52" s="16"/>
+      <c r="C52" s="56" t="s">
         <v>95</v>
       </c>
-      <c r="D51" s="66"/>
-    </row>
-    <row r="52" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B52" s="16"/>
-      <c r="C52" s="65" t="s">
+      <c r="D52" s="57"/>
+    </row>
+    <row r="54" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B54" s="63" t="s">
         <v>96</v>
       </c>
-      <c r="D52" s="66"/>
-    </row>
-    <row r="54" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B54" s="60" t="s">
-        <v>97</v>
-      </c>
-      <c r="C54" s="61"/>
-      <c r="D54" s="61"/>
-      <c r="E54" s="53" t="s">
-        <v>92</v>
-      </c>
-      <c r="F54" s="53"/>
-      <c r="G54" s="53"/>
-      <c r="H54" s="53"/>
-    </row>
-    <row r="55" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C54" s="64"/>
+      <c r="D54" s="64"/>
+      <c r="E54" s="62" t="s">
+        <v>91</v>
+      </c>
+      <c r="F54" s="62"/>
+      <c r="G54" s="62"/>
+      <c r="H54" s="62"/>
+    </row>
+    <row r="55" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B55" s="47" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C55" s="47" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D55" s="47" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E55" s="51" t="s">
+        <v>87</v>
+      </c>
+      <c r="F55" s="51" t="s">
         <v>88</v>
       </c>
-      <c r="F55" s="51" t="s">
+      <c r="G55" s="51" t="s">
         <v>89</v>
       </c>
-      <c r="G55" s="51" t="s">
+      <c r="H55" s="51" t="s">
         <v>90</v>
       </c>
-      <c r="H55" s="51" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="56" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="56" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B56">
         <v>1</v>
       </c>
       <c r="C56" s="36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D56" s="36" t="s">
         <v>19</v>
-      </c>
-      <c r="D56" s="36" t="s">
-        <v>20</v>
       </c>
       <c r="E56" s="2">
         <v>196363.85601577908</v>
@@ -3452,15 +3339,15 @@
         <v>291463.48739316239</v>
       </c>
     </row>
-    <row r="57" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B57">
         <v>2</v>
       </c>
       <c r="C57" s="36" t="s">
+        <v>20</v>
+      </c>
+      <c r="D57" t="s">
         <v>21</v>
-      </c>
-      <c r="D57" t="s">
-        <v>22</v>
       </c>
       <c r="E57" s="2">
         <v>141843.80341880341</v>
@@ -3475,15 +3362,15 @@
         <v>243711.7393984221</v>
       </c>
     </row>
-    <row r="58" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B58">
         <v>3</v>
       </c>
       <c r="C58" s="36" t="s">
+        <v>22</v>
+      </c>
+      <c r="D58" t="s">
         <v>23</v>
-      </c>
-      <c r="D58" t="s">
-        <v>24</v>
       </c>
       <c r="E58" s="2">
         <v>92775.756081525309</v>
@@ -3498,15 +3385,15 @@
         <v>171882.31025641024</v>
       </c>
     </row>
-    <row r="59" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B59">
         <v>4</v>
       </c>
       <c r="C59" s="36" t="s">
+        <v>24</v>
+      </c>
+      <c r="D59" t="s">
         <v>25</v>
-      </c>
-      <c r="D59" t="s">
-        <v>26</v>
       </c>
       <c r="E59" s="2">
         <v>103679.76660092045</v>
@@ -3521,15 +3408,15 @@
         <v>174043.68658229234</v>
       </c>
     </row>
-    <row r="60" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B60">
         <v>5</v>
       </c>
       <c r="C60" s="36" t="s">
+        <v>26</v>
+      </c>
+      <c r="D60" t="s">
         <v>27</v>
-      </c>
-      <c r="D60" t="s">
-        <v>28</v>
       </c>
       <c r="E60" s="2">
         <v>109131.77186061803</v>
@@ -3544,15 +3431,15 @@
         <v>186127.86278216087</v>
       </c>
     </row>
-    <row r="61" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B61">
         <v>6</v>
       </c>
       <c r="C61" t="s">
+        <v>28</v>
+      </c>
+      <c r="D61" t="s">
         <v>29</v>
-      </c>
-      <c r="D61" t="s">
-        <v>30</v>
       </c>
       <c r="E61" s="2">
         <v>70967.735042735047</v>
@@ -3567,15 +3454,15 @@
         <v>77347.585968660962</v>
       </c>
     </row>
-    <row r="62" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B62">
         <v>7</v>
       </c>
       <c r="C62" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D62" s="36" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E62" s="2">
         <v>45888.510848126229</v>
@@ -3590,15 +3477,15 @@
         <v>56250.410693622624</v>
       </c>
     </row>
-    <row r="63" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B63">
         <v>8</v>
       </c>
       <c r="C63" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D63" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E63" s="2">
         <v>49159.71400394477</v>
@@ -3613,15 +3500,15 @@
         <v>98676.840581854049</v>
       </c>
     </row>
-    <row r="64" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B64">
         <v>9</v>
       </c>
       <c r="C64" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D64" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E64" s="2">
         <v>54611.71926364235</v>
@@ -3636,15 +3523,15 @@
         <v>79000.307774490459</v>
       </c>
     </row>
-    <row r="65" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B65">
         <v>10</v>
       </c>
       <c r="C65" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D65" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E65" s="2">
         <v>29532.495069033528</v>
@@ -3659,15 +3546,15 @@
         <v>40857.773875739644</v>
       </c>
     </row>
-    <row r="66" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B66">
         <v>11</v>
       </c>
       <c r="C66" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D66" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E66" s="2">
         <v>24080.489809335966</v>
@@ -3682,15 +3569,15 @@
         <v>28705.43665680473</v>
       </c>
     </row>
-    <row r="67" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B67">
         <v>12</v>
       </c>
       <c r="C67" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D67" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E67" s="2">
         <v>27351.692965154507</v>
@@ -3705,15 +3592,15 @@
         <v>41302.205374753452</v>
       </c>
     </row>
-    <row r="68" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B68">
         <v>13</v>
       </c>
       <c r="C68" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D68" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E68" s="2">
         <v>28442.094017094016</v>
@@ -3728,15 +3615,15 @@
         <v>52090.041182336165</v>
       </c>
     </row>
-    <row r="69" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B69">
         <v>14</v>
       </c>
       <c r="C69" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D69" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E69" s="2">
         <v>15357.281393819854</v>
@@ -3751,15 +3638,15 @@
         <v>17209.08684089415</v>
       </c>
     </row>
-    <row r="70" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B70">
         <v>15</v>
       </c>
       <c r="C70" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D70" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E70" s="2">
         <v>13176.479289940828</v>
@@ -3774,15 +3661,15 @@
         <v>20834.274151873768</v>
       </c>
     </row>
-    <row r="71" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B71">
         <v>16</v>
       </c>
       <c r="C71" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D71" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E71" s="2">
         <v>27351.692965154507</v>
@@ -3797,15 +3684,15 @@
         <v>49035.369466359865</v>
       </c>
     </row>
-    <row r="72" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B72">
         <v>17</v>
       </c>
       <c r="C72" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D72" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E72" s="2">
         <v>32803.698224852073</v>
@@ -3820,15 +3707,15 @@
         <v>42936.122994740297</v>
       </c>
     </row>
-    <row r="73" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B73">
         <v>18</v>
       </c>
       <c r="C73" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D73" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E73" s="2">
         <v>43707.708744247211</v>
@@ -3843,15 +3730,15 @@
         <v>70319.545666228354</v>
       </c>
     </row>
-    <row r="74" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B74">
         <v>19</v>
       </c>
       <c r="C74" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D74" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E74" s="2">
         <v>45888.510848126229</v>
@@ -3866,15 +3753,15 @@
         <v>63593.453862590402</v>
       </c>
     </row>
-    <row r="75" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B75">
         <v>20</v>
       </c>
       <c r="C75" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D75" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E75" s="2">
         <v>30622.896120973044</v>
@@ -3889,9 +3776,9 @@
         <v>32447.5589031339</v>
       </c>
     </row>
-    <row r="78" spans="2:8" ht="23.4" x14ac:dyDescent="0.45">
+    <row r="78" spans="2:8" ht="24" x14ac:dyDescent="0.3">
       <c r="B78" s="25" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C78" s="1"/>
       <c r="D78" s="1"/>
@@ -3899,74 +3786,74 @@
       <c r="F78" s="1"/>
       <c r="G78" s="1"/>
     </row>
-    <row r="79" spans="2:8" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="79" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B79" s="18"/>
     </row>
-    <row r="80" spans="2:8" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="80" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B80" s="52" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C80" s="1"/>
       <c r="D80" s="37"/>
       <c r="E80" s="37"/>
       <c r="F80" s="37"/>
     </row>
-    <row r="81" spans="2:46" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="81" spans="2:46" x14ac:dyDescent="0.2">
       <c r="B81" s="46"/>
-      <c r="C81" s="65" t="s">
+      <c r="C81" s="56" t="s">
+        <v>93</v>
+      </c>
+      <c r="D81" s="57"/>
+      <c r="E81" s="57"/>
+      <c r="F81" s="57"/>
+    </row>
+    <row r="82" spans="2:46" x14ac:dyDescent="0.2">
+      <c r="B82" s="15"/>
+      <c r="C82" s="56" t="s">
         <v>94</v>
       </c>
-      <c r="D81" s="66"/>
-      <c r="E81" s="66"/>
-      <c r="F81" s="66"/>
-    </row>
-    <row r="82" spans="2:46" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B82" s="15"/>
-      <c r="C82" s="65" t="s">
+      <c r="D82" s="57"/>
+      <c r="E82" s="57"/>
+      <c r="F82" s="57"/>
+    </row>
+    <row r="83" spans="2:46" x14ac:dyDescent="0.2">
+      <c r="B83" s="16"/>
+      <c r="C83" s="56" t="s">
         <v>95</v>
       </c>
-      <c r="D82" s="66"/>
-      <c r="E82" s="66"/>
-      <c r="F82" s="66"/>
-    </row>
-    <row r="83" spans="2:46" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B83" s="16"/>
-      <c r="C83" s="65" t="s">
-        <v>96</v>
-      </c>
-      <c r="D83" s="66"/>
-      <c r="E83" s="66"/>
-      <c r="F83" s="66"/>
-    </row>
-    <row r="84" spans="2:46" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="D83" s="57"/>
+      <c r="E83" s="57"/>
+      <c r="F83" s="57"/>
+    </row>
+    <row r="84" spans="2:46" x14ac:dyDescent="0.2">
       <c r="AR84" s="3"/>
       <c r="AS84" s="3"/>
       <c r="AT84" s="3"/>
     </row>
-    <row r="85" spans="2:46" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B85" s="60" t="s">
-        <v>97</v>
-      </c>
-      <c r="C85" s="61"/>
-      <c r="D85" s="61"/>
-      <c r="E85" s="63" t="s">
-        <v>73</v>
-      </c>
-      <c r="F85" s="63"/>
-      <c r="G85" s="63"/>
-      <c r="H85" s="63"/>
-      <c r="I85" s="62" t="s">
-        <v>82</v>
-      </c>
-      <c r="J85" s="62"/>
-      <c r="K85" s="62"/>
-      <c r="L85" s="62"/>
-      <c r="M85" s="64" t="s">
-        <v>87</v>
-      </c>
-      <c r="N85" s="64"/>
-      <c r="O85" s="64"/>
-      <c r="P85" s="64"/>
+    <row r="85" spans="2:46" x14ac:dyDescent="0.2">
+      <c r="B85" s="63" t="s">
+        <v>96</v>
+      </c>
+      <c r="C85" s="64"/>
+      <c r="D85" s="64"/>
+      <c r="E85" s="65" t="s">
+        <v>72</v>
+      </c>
+      <c r="F85" s="65"/>
+      <c r="G85" s="65"/>
+      <c r="H85" s="65"/>
+      <c r="I85" s="67" t="s">
+        <v>81</v>
+      </c>
+      <c r="J85" s="67"/>
+      <c r="K85" s="67"/>
+      <c r="L85" s="67"/>
+      <c r="M85" s="66" t="s">
+        <v>86</v>
+      </c>
+      <c r="N85" s="66"/>
+      <c r="O85" s="66"/>
+      <c r="P85" s="66"/>
       <c r="U85" s="31"/>
       <c r="V85" s="31"/>
       <c r="W85" s="31"/>
@@ -3977,51 +3864,51 @@
       <c r="AB85" s="31"/>
       <c r="AC85" s="31"/>
     </row>
-    <row r="86" spans="2:46" ht="24" x14ac:dyDescent="0.3">
+    <row r="86" spans="2:46" ht="28" x14ac:dyDescent="0.2">
       <c r="B86" s="47" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C86" s="47" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D86" s="47" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E86" s="48" t="s">
+        <v>73</v>
+      </c>
+      <c r="F86" s="48" t="s">
         <v>74</v>
       </c>
-      <c r="F86" s="48" t="s">
+      <c r="G86" s="48" t="s">
         <v>75</v>
       </c>
-      <c r="G86" s="48" t="s">
+      <c r="H86" s="48" t="s">
         <v>76</v>
       </c>
-      <c r="H86" s="48" t="s">
+      <c r="I86" s="49" t="s">
         <v>77</v>
       </c>
-      <c r="I86" s="49" t="s">
+      <c r="J86" s="49" t="s">
         <v>78</v>
       </c>
-      <c r="J86" s="49" t="s">
+      <c r="K86" s="49" t="s">
         <v>79</v>
       </c>
-      <c r="K86" s="49" t="s">
+      <c r="L86" s="49" t="s">
         <v>80</v>
       </c>
-      <c r="L86" s="49" t="s">
-        <v>81</v>
-      </c>
       <c r="M86" s="50" t="s">
+        <v>82</v>
+      </c>
+      <c r="N86" s="50" t="s">
         <v>83</v>
       </c>
-      <c r="N86" s="50" t="s">
+      <c r="O86" s="50" t="s">
         <v>84</v>
       </c>
-      <c r="O86" s="50" t="s">
+      <c r="P86" s="50" t="s">
         <v>85</v>
-      </c>
-      <c r="P86" s="50" t="s">
-        <v>86</v>
       </c>
       <c r="U86" s="32"/>
       <c r="V86" s="32"/>
@@ -4034,15 +3921,15 @@
       <c r="AC86" s="32"/>
       <c r="AF86" s="33"/>
     </row>
-    <row r="87" spans="2:46" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:46" ht="16" x14ac:dyDescent="0.2">
       <c r="B87">
         <v>1</v>
       </c>
       <c r="C87" s="36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D87" s="36" t="s">
         <v>19</v>
-      </c>
-      <c r="D87" s="36" t="s">
-        <v>20</v>
       </c>
       <c r="E87" s="2">
         <v>1677000</v>
@@ -4082,15 +3969,15 @@
       </c>
       <c r="AF87" s="31"/>
     </row>
-    <row r="88" spans="2:46" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="88" spans="2:46" ht="16" x14ac:dyDescent="0.2">
       <c r="B88">
         <v>2</v>
       </c>
       <c r="C88" s="36" t="s">
+        <v>20</v>
+      </c>
+      <c r="D88" t="s">
         <v>21</v>
-      </c>
-      <c r="D88" t="s">
-        <v>22</v>
       </c>
       <c r="E88" s="2">
         <v>1440000</v>
@@ -4130,15 +4017,15 @@
       </c>
       <c r="AF88" s="33"/>
     </row>
-    <row r="89" spans="2:46" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="89" spans="2:46" ht="16" x14ac:dyDescent="0.2">
       <c r="B89">
         <v>3</v>
       </c>
       <c r="C89" s="36" t="s">
+        <v>22</v>
+      </c>
+      <c r="D89" t="s">
         <v>23</v>
-      </c>
-      <c r="D89" t="s">
-        <v>24</v>
       </c>
       <c r="E89" s="2">
         <v>994500</v>
@@ -4177,15 +4064,15 @@
         <v>2062587.7230769231</v>
       </c>
     </row>
-    <row r="90" spans="2:46" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="90" spans="2:46" ht="16" x14ac:dyDescent="0.2">
       <c r="B90">
         <v>4</v>
       </c>
       <c r="C90" s="36" t="s">
+        <v>24</v>
+      </c>
+      <c r="D90" t="s">
         <v>25</v>
-      </c>
-      <c r="D90" t="s">
-        <v>26</v>
       </c>
       <c r="E90" s="2">
         <v>950000</v>
@@ -4224,15 +4111,15 @@
         <v>2088524.2389875082</v>
       </c>
     </row>
-    <row r="91" spans="2:46" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="91" spans="2:46" ht="16" x14ac:dyDescent="0.2">
       <c r="B91">
         <v>5</v>
       </c>
       <c r="C91" s="36" t="s">
+        <v>26</v>
+      </c>
+      <c r="D91" t="s">
         <v>27</v>
-      </c>
-      <c r="D91" t="s">
-        <v>28</v>
       </c>
       <c r="E91" s="2">
         <v>1070000</v>
@@ -4271,15 +4158,15 @@
         <v>2233534.3533859304</v>
       </c>
     </row>
-    <row r="92" spans="2:46" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="92" spans="2:46" x14ac:dyDescent="0.2">
       <c r="B92">
         <v>6</v>
       </c>
       <c r="C92" t="s">
+        <v>28</v>
+      </c>
+      <c r="D92" t="s">
         <v>29</v>
-      </c>
-      <c r="D92" t="s">
-        <v>30</v>
       </c>
       <c r="E92" s="2">
         <v>461500</v>
@@ -4318,15 +4205,15 @@
         <v>928171.0316239316</v>
       </c>
     </row>
-    <row r="93" spans="2:46" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="93" spans="2:46" ht="16" x14ac:dyDescent="0.2">
       <c r="B93">
         <v>7</v>
       </c>
       <c r="C93" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D93" s="36" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E93" s="2">
         <v>344400</v>
@@ -4365,15 +4252,15 @@
         <v>675004.92832347145</v>
       </c>
     </row>
-    <row r="94" spans="2:46" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="94" spans="2:46" x14ac:dyDescent="0.2">
       <c r="B94">
         <v>8</v>
       </c>
       <c r="C94" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D94" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E94" s="2">
         <v>589500</v>
@@ -4412,15 +4299,15 @@
         <v>1184122.0869822486</v>
       </c>
     </row>
-    <row r="95" spans="2:46" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="95" spans="2:46" x14ac:dyDescent="0.2">
       <c r="B95">
         <v>9</v>
       </c>
       <c r="C95" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D95" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E95" s="2">
         <v>465000</v>
@@ -4459,15 +4346,15 @@
         <v>948003.69329388556</v>
       </c>
     </row>
-    <row r="96" spans="2:46" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="96" spans="2:46" x14ac:dyDescent="0.2">
       <c r="B96">
         <v>10</v>
       </c>
       <c r="C96" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D96" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E96" s="2">
         <v>237600</v>
@@ -4506,15 +4393,15 @@
         <v>490293.28650887572</v>
       </c>
     </row>
-    <row r="97" spans="2:16" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="97" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B97">
         <v>11</v>
       </c>
       <c r="C97" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D97" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E97" s="2">
         <v>178200</v>
@@ -4553,15 +4440,15 @@
         <v>344465.23988165677</v>
       </c>
     </row>
-    <row r="98" spans="2:16" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="98" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B98">
         <v>12</v>
       </c>
       <c r="C98" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D98" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E98" s="2">
         <v>225000</v>
@@ -4600,15 +4487,15 @@
         <v>495626.46449704142</v>
       </c>
     </row>
-    <row r="99" spans="2:16" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="99" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B99">
         <v>13</v>
       </c>
       <c r="C99" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D99" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E99" s="2">
         <v>301599.99999999994</v>
@@ -4647,15 +4534,15 @@
         <v>625080.49418803398</v>
       </c>
     </row>
-    <row r="100" spans="2:16" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="100" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B100">
         <v>14</v>
       </c>
       <c r="C100" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D100" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E100" s="2">
         <v>96600</v>
@@ -4694,15 +4581,15 @@
         <v>206509.04209072978</v>
       </c>
     </row>
-    <row r="101" spans="2:16" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="101" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B101">
         <v>15</v>
       </c>
       <c r="C101" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D101" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E101" s="2">
         <v>115200</v>
@@ -4741,15 +4628,15 @@
         <v>250011.28982248521</v>
       </c>
     </row>
-    <row r="102" spans="2:16" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="102" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B102">
         <v>16</v>
       </c>
       <c r="C102" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D102" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E102" s="2">
         <v>280000.00000000006</v>
@@ -4788,15 +4675,15 @@
         <v>588424.43359631835</v>
       </c>
     </row>
-    <row r="103" spans="2:16" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="103" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B103">
         <v>17</v>
       </c>
       <c r="C103" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D103" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E103" s="2">
         <v>237000</v>
@@ -4835,15 +4722,15 @@
         <v>515233.47593688359</v>
       </c>
     </row>
-    <row r="104" spans="2:16" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="104" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B104">
         <v>18</v>
       </c>
       <c r="C104" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D104" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E104" s="2">
         <v>400000</v>
@@ -4882,15 +4769,15 @@
         <v>843834.54799474031</v>
       </c>
     </row>
-    <row r="105" spans="2:16" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="105" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B105">
         <v>19</v>
       </c>
       <c r="C105" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D105" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E105" s="2">
         <v>373800</v>
@@ -4929,15 +4816,15 @@
         <v>763121.44635108486</v>
       </c>
     </row>
-    <row r="106" spans="2:16" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="106" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B106">
         <v>20</v>
       </c>
       <c r="C106" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D106" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E106" s="2">
         <v>182000</v>
@@ -4976,75 +4863,75 @@
         <v>389370.70683760679</v>
       </c>
     </row>
-    <row r="107" spans="2:16" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="108" spans="2:16" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="109" spans="2:16" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="110" spans="2:16" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="111" spans="2:16" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="112" spans="2:16" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="113" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="114" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="115" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="116" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="117" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="118" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="119" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="120" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="121" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="122" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="123" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="124" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="125" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="126" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="127" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="128" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="129" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="130" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="131" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="132" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="133" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="134" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="135" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="136" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="137" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="138" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="139" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="140" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="141" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="142" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="143" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="144" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="145" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="146" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="147" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="148" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="149" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="150" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="151" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="152" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="153" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="154" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="155" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="156" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="157" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="158" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="159" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="160" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="161" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="162" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="163" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="164" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="165" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="166" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="167" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="168" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="169" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="170" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="171" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="172" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="173" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="174" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="175" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="107" spans="2:16" x14ac:dyDescent="0.2"/>
+    <row r="108" spans="2:16" x14ac:dyDescent="0.2"/>
+    <row r="109" spans="2:16" x14ac:dyDescent="0.2"/>
+    <row r="110" spans="2:16" x14ac:dyDescent="0.2"/>
+    <row r="111" spans="2:16" x14ac:dyDescent="0.2"/>
+    <row r="112" spans="2:16" x14ac:dyDescent="0.2"/>
+    <row r="113" x14ac:dyDescent="0.2"/>
+    <row r="114" x14ac:dyDescent="0.2"/>
+    <row r="115" x14ac:dyDescent="0.2"/>
+    <row r="116" x14ac:dyDescent="0.2"/>
+    <row r="117" x14ac:dyDescent="0.2"/>
+    <row r="118" x14ac:dyDescent="0.2"/>
+    <row r="119" x14ac:dyDescent="0.2"/>
+    <row r="120" x14ac:dyDescent="0.2"/>
+    <row r="121" x14ac:dyDescent="0.2"/>
+    <row r="122" x14ac:dyDescent="0.2"/>
+    <row r="123" x14ac:dyDescent="0.2"/>
+    <row r="124" x14ac:dyDescent="0.2"/>
+    <row r="125" x14ac:dyDescent="0.2"/>
+    <row r="126" x14ac:dyDescent="0.2"/>
+    <row r="127" x14ac:dyDescent="0.2"/>
+    <row r="128" x14ac:dyDescent="0.2"/>
+    <row r="129" x14ac:dyDescent="0.2"/>
+    <row r="130" x14ac:dyDescent="0.2"/>
+    <row r="131" x14ac:dyDescent="0.2"/>
+    <row r="132" x14ac:dyDescent="0.2"/>
+    <row r="133" x14ac:dyDescent="0.2"/>
+    <row r="134" x14ac:dyDescent="0.2"/>
+    <row r="135" x14ac:dyDescent="0.2"/>
+    <row r="136" x14ac:dyDescent="0.2"/>
+    <row r="137" x14ac:dyDescent="0.2"/>
+    <row r="138" x14ac:dyDescent="0.2"/>
+    <row r="139" x14ac:dyDescent="0.2"/>
+    <row r="140" x14ac:dyDescent="0.2"/>
+    <row r="141" x14ac:dyDescent="0.2"/>
+    <row r="142" x14ac:dyDescent="0.2"/>
+    <row r="143" x14ac:dyDescent="0.2"/>
+    <row r="144" x14ac:dyDescent="0.2"/>
+    <row r="145" x14ac:dyDescent="0.2"/>
+    <row r="146" x14ac:dyDescent="0.2"/>
+    <row r="147" x14ac:dyDescent="0.2"/>
+    <row r="148" x14ac:dyDescent="0.2"/>
+    <row r="149" x14ac:dyDescent="0.2"/>
+    <row r="150" x14ac:dyDescent="0.2"/>
+    <row r="151" x14ac:dyDescent="0.2"/>
+    <row r="152" x14ac:dyDescent="0.2"/>
+    <row r="153" x14ac:dyDescent="0.2"/>
+    <row r="154" x14ac:dyDescent="0.2"/>
+    <row r="155" x14ac:dyDescent="0.2"/>
+    <row r="156" x14ac:dyDescent="0.2"/>
+    <row r="157" x14ac:dyDescent="0.2"/>
+    <row r="158" x14ac:dyDescent="0.2"/>
+    <row r="159" x14ac:dyDescent="0.2"/>
+    <row r="160" x14ac:dyDescent="0.2"/>
+    <row r="161" x14ac:dyDescent="0.2"/>
+    <row r="162" x14ac:dyDescent="0.2"/>
+    <row r="163" x14ac:dyDescent="0.2"/>
+    <row r="164" x14ac:dyDescent="0.2"/>
+    <row r="165" x14ac:dyDescent="0.2"/>
+    <row r="166" x14ac:dyDescent="0.2"/>
+    <row r="167" x14ac:dyDescent="0.2"/>
+    <row r="168" x14ac:dyDescent="0.2"/>
+    <row r="169" x14ac:dyDescent="0.2"/>
+    <row r="170" x14ac:dyDescent="0.2"/>
+    <row r="171" x14ac:dyDescent="0.2"/>
+    <row r="172" x14ac:dyDescent="0.2"/>
+    <row r="173" x14ac:dyDescent="0.2"/>
+    <row r="174" x14ac:dyDescent="0.2"/>
+    <row r="175" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="19">
     <mergeCell ref="B85:D85"/>
@@ -5053,26 +4940,25 @@
     <mergeCell ref="I85:L85"/>
     <mergeCell ref="C81:F81"/>
     <mergeCell ref="C82:F82"/>
+    <mergeCell ref="B37:G37"/>
+    <mergeCell ref="C83:F83"/>
+    <mergeCell ref="B4:AO4"/>
+    <mergeCell ref="B15:G19"/>
+    <mergeCell ref="B20:G21"/>
+    <mergeCell ref="B27:G28"/>
+    <mergeCell ref="B30:G31"/>
     <mergeCell ref="B40:G41"/>
     <mergeCell ref="C50:D50"/>
     <mergeCell ref="C51:D51"/>
     <mergeCell ref="C52:D52"/>
     <mergeCell ref="E54:H54"/>
     <mergeCell ref="B54:D54"/>
-    <mergeCell ref="B4:AO4"/>
-    <mergeCell ref="B15:G19"/>
-    <mergeCell ref="B20:G21"/>
-    <mergeCell ref="B27:G28"/>
-    <mergeCell ref="B30:G31"/>
-    <mergeCell ref="B37:G37"/>
-    <mergeCell ref="C83:F83"/>
   </mergeCells>
   <phoneticPr fontId="25" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
   <tableParts count="2">
+    <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
-    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>